<commit_message>
Sprint 5 Day 32: Capital Allocation Report implemented
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -512,11 +512,7 @@
       <c r="J2" t="b">
         <v>1</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -557,11 +553,7 @@
       <c r="J3" t="b">
         <v>0</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -602,11 +594,7 @@
       <c r="J4" t="b">
         <v>0</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -647,11 +635,7 @@
       <c r="J5" t="b">
         <v>0</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -692,11 +676,7 @@
       <c r="J6" t="b">
         <v>0</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -737,11 +717,7 @@
       <c r="J7" t="b">
         <v>0</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -782,11 +758,7 @@
       <c r="J8" t="b">
         <v>0</v>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -827,11 +799,7 @@
       <c r="J9" t="b">
         <v>0</v>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -872,11 +840,7 @@
       <c r="J10" t="b">
         <v>0</v>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -915,11 +879,7 @@
       <c r="J11" t="b">
         <v>0</v>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -960,11 +920,7 @@
       <c r="J12" t="b">
         <v>0</v>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1005,11 +961,7 @@
       <c r="J13" t="b">
         <v>0</v>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1050,11 +1002,7 @@
       <c r="J14" t="b">
         <v>0</v>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1095,11 +1043,7 @@
       <c r="J15" t="b">
         <v>1</v>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1140,11 +1084,7 @@
       <c r="J16" t="b">
         <v>0</v>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1185,11 +1125,7 @@
       <c r="J17" t="b">
         <v>0</v>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1230,11 +1166,7 @@
       <c r="J18" t="b">
         <v>0</v>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1275,11 +1207,7 @@
       <c r="J19" t="b">
         <v>0</v>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1320,11 +1248,7 @@
       <c r="J20" t="b">
         <v>0</v>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1365,11 +1289,7 @@
       <c r="J21" t="b">
         <v>1</v>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1410,11 +1330,7 @@
       <c r="J22" t="b">
         <v>0</v>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1455,11 +1371,7 @@
       <c r="J23" t="b">
         <v>0</v>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1500,11 +1412,7 @@
       <c r="J24" t="b">
         <v>0</v>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1545,11 +1453,7 @@
       <c r="J25" t="b">
         <v>0</v>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1590,11 +1494,7 @@
       <c r="J26" t="b">
         <v>1</v>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1635,11 +1535,7 @@
       <c r="J27" t="b">
         <v>0</v>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1680,11 +1576,7 @@
       <c r="J28" t="b">
         <v>0</v>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1725,11 +1617,7 @@
       <c r="J29" t="b">
         <v>0</v>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1770,11 +1658,7 @@
       <c r="J30" t="b">
         <v>0</v>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1815,11 +1699,7 @@
       <c r="J31" t="b">
         <v>0</v>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1860,11 +1740,7 @@
       <c r="J32" t="b">
         <v>0</v>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1905,11 +1781,7 @@
       <c r="J33" t="b">
         <v>1</v>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1950,11 +1822,7 @@
       <c r="J34" t="b">
         <v>1</v>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1995,11 +1863,7 @@
       <c r="J35" t="b">
         <v>0</v>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2040,11 +1904,7 @@
       <c r="J36" t="b">
         <v>0</v>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2085,11 +1945,7 @@
       <c r="J37" t="b">
         <v>0</v>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2130,11 +1986,7 @@
       <c r="J38" t="b">
         <v>0</v>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2175,11 +2027,7 @@
       <c r="J39" t="b">
         <v>0</v>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2220,11 +2068,7 @@
       <c r="J40" t="b">
         <v>0</v>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2265,11 +2109,7 @@
       <c r="J41" t="b">
         <v>0</v>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2310,11 +2150,7 @@
       <c r="J42" t="b">
         <v>1</v>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2355,11 +2191,7 @@
       <c r="J43" t="b">
         <v>0</v>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2400,11 +2232,7 @@
       <c r="J44" t="b">
         <v>0</v>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2445,11 +2273,7 @@
       <c r="J45" t="b">
         <v>0</v>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2490,11 +2314,7 @@
       <c r="J46" t="b">
         <v>1</v>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2535,11 +2355,7 @@
       <c r="J47" t="b">
         <v>1</v>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2580,11 +2396,7 @@
       <c r="J48" t="b">
         <v>0</v>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2625,11 +2437,7 @@
       <c r="J49" t="b">
         <v>0</v>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2670,11 +2478,7 @@
       <c r="J50" t="b">
         <v>0</v>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2715,11 +2519,7 @@
       <c r="J51" t="b">
         <v>0</v>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2760,11 +2560,7 @@
       <c r="J52" t="b">
         <v>1</v>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2805,11 +2601,7 @@
       <c r="J53" t="b">
         <v>1</v>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2850,11 +2642,7 @@
       <c r="J54" t="b">
         <v>0</v>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2895,11 +2683,7 @@
       <c r="J55" t="b">
         <v>0</v>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2940,11 +2724,7 @@
       <c r="J56" t="b">
         <v>0</v>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2985,11 +2765,7 @@
       <c r="J57" t="b">
         <v>0</v>
       </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3030,11 +2806,7 @@
       <c r="J58" t="b">
         <v>0</v>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3075,11 +2847,7 @@
       <c r="J59" t="b">
         <v>0</v>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3120,11 +2888,7 @@
       <c r="J60" t="b">
         <v>0</v>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3165,11 +2929,7 @@
       <c r="J61" t="b">
         <v>0</v>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3210,11 +2970,7 @@
       <c r="J62" t="b">
         <v>0</v>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3255,11 +3011,7 @@
       <c r="J63" t="b">
         <v>0</v>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3300,11 +3052,7 @@
       <c r="J64" t="b">
         <v>0</v>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3345,11 +3093,7 @@
       <c r="J65" t="b">
         <v>0</v>
       </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3390,11 +3134,7 @@
       <c r="J66" t="b">
         <v>0</v>
       </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3435,11 +3175,7 @@
       <c r="J67" t="b">
         <v>0</v>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3480,11 +3216,7 @@
       <c r="J68" t="b">
         <v>0</v>
       </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3525,11 +3257,7 @@
       <c r="J69" t="b">
         <v>0</v>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3570,11 +3298,7 @@
       <c r="J70" t="b">
         <v>0</v>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3615,11 +3339,7 @@
       <c r="J71" t="b">
         <v>0</v>
       </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3660,11 +3380,7 @@
       <c r="J72" t="b">
         <v>0</v>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3705,11 +3421,7 @@
       <c r="J73" t="b">
         <v>1</v>
       </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3750,11 +3462,7 @@
       <c r="J74" t="b">
         <v>0</v>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3795,11 +3503,7 @@
       <c r="J75" t="b">
         <v>0</v>
       </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3840,11 +3544,7 @@
       <c r="J76" t="b">
         <v>0</v>
       </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3885,11 +3585,7 @@
       <c r="J77" t="b">
         <v>1</v>
       </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3930,11 +3626,7 @@
       <c r="J78" t="b">
         <v>0</v>
       </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3975,11 +3667,7 @@
       <c r="J79" t="b">
         <v>0</v>
       </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4020,11 +3708,7 @@
       <c r="J80" t="b">
         <v>0</v>
       </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4067,7 +3751,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Cash Cow</t>
+          <t>Cash Cow / Self-Sustaining</t>
         </is>
       </c>
     </row>
@@ -4110,11 +3794,7 @@
       <c r="J82" t="b">
         <v>1</v>
       </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4155,11 +3835,7 @@
       <c r="J83" t="b">
         <v>0</v>
       </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4200,11 +3876,7 @@
       <c r="J84" t="b">
         <v>1</v>
       </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4245,11 +3917,7 @@
       <c r="J85" t="b">
         <v>0</v>
       </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>Aggressive Growth</t>
-        </is>
-      </c>
+      <c r="K85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4290,11 +3958,7 @@
       <c r="J86" t="b">
         <v>0</v>
       </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4335,11 +3999,7 @@
       <c r="J87" t="b">
         <v>0</v>
       </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4380,11 +4040,7 @@
       <c r="J88" t="b">
         <v>0</v>
       </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4425,11 +4081,7 @@
       <c r="J89" t="b">
         <v>0</v>
       </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4470,11 +4122,7 @@
       <c r="J90" t="b">
         <v>1</v>
       </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
+      <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4515,11 +4163,7 @@
       <c r="J91" t="b">
         <v>0</v>
       </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>Self-Sustaining</t>
-        </is>
-      </c>
+      <c r="K91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4560,11 +4204,7 @@
       <c r="J92" t="b">
         <v>0</v>
       </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>External Dependent</t>
-        </is>
-      </c>
+      <c r="K92" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>